<commit_message>
docs(registration): finalize all member details for Nafiz and Anona in registration sheet and submission package
</commit_message>
<xml_diff>
--- a/submission_package/Registration_Form_AegisPay_Filled.xlsx
+++ b/submission_package/Registration_Form_AegisPay_Filled.xlsx
@@ -952,7 +952,7 @@
       </c>
       <c r="N11" s="25" t="inlineStr">
         <is>
-          <t>+60 12-345 6789</t>
+          <t>+8801515636528</t>
         </is>
       </c>
     </row>
@@ -985,14 +985,44 @@
           <t>Passport</t>
         </is>
       </c>
-      <c r="G12" s="19" t="n"/>
-      <c r="H12" s="19" t="n"/>
-      <c r="I12" s="19" t="n"/>
-      <c r="J12" s="19" t="n"/>
-      <c r="K12" s="19" t="n"/>
-      <c r="L12" t="inlineStr">
+      <c r="G12" s="19" t="inlineStr">
+        <is>
+          <t>A05592099</t>
+        </is>
+      </c>
+      <c r="H12" s="19" t="inlineStr">
+        <is>
+          <t>0432220005101011</t>
+        </is>
+      </c>
+      <c r="I12" s="19" t="inlineStr">
+        <is>
+          <t>University of Information Technology and Sciences</t>
+        </is>
+      </c>
+      <c r="J12" s="19" t="inlineStr">
+        <is>
+          <t>Computer Science and Engineering</t>
+        </is>
+      </c>
+      <c r="K12" s="19" t="inlineStr">
+        <is>
+          <t>UG Year 4</t>
+        </is>
+      </c>
+      <c r="L12" s="12" t="inlineStr">
         <is>
           <t>student_card_Anona_Ayshi_Rozario.pdf</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>0432220005101011@uits.edu.bd</t>
+        </is>
+      </c>
+      <c r="N12" s="12" t="inlineStr">
+        <is>
+          <t>+8801554164137</t>
         </is>
       </c>
     </row>

</xml_diff>